<commit_message>
fix: stock/inventory writes now target the fields checkout reads
- adminCreateProduct/adminUpdateProduct: whitelist top-level stock so
  the Add/Edit Product form can persist it
- adminUpdateInventory: write to stock/variants[].stock instead of
  stores[], which checkout never reads
- bulk upload: read a real stock value from the uploaded file instead
  of hardcoding every variant to 0; add stock column to the product
  upload template
- admin.js: add Stock field to Add/Edit Product modal
</commit_message>
<xml_diff>
--- a/frontend/nc_assets/files/Sagona_Product_Upload_Template.xlsx
+++ b/frontend/nc_assets/files/Sagona_Product_Upload_Template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Measurements" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -188,7 +188,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -241,6 +241,9 @@
     <xf numFmtId="0" fontId="12" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -606,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -629,6 +632,7 @@
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -739,6 +743,11 @@
           <t>hsn_code</t>
         </is>
       </c>
+      <c r="U2" s="19" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -839,6 +848,11 @@
       <c r="T3" s="4" t="inlineStr">
         <is>
           <t>GST HSN code</t>
+        </is>
+      </c>
+      <c r="U3" s="20" t="inlineStr">
+        <is>
+          <t>Available quantity (0 if blank). Applied to every size/colour combo if variants used</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1158,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A1:U1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1693,7 +1707,7 @@
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Stock quantities start at 0 — update them via product Inventory after upload</t>
+          <t xml:space="preserve">  • Stock: set the stock column per product (applied to every size/colour combo for variant products). Leave blank for 0.</t>
         </is>
       </c>
     </row>
@@ -1730,8 +1744,8 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A23:B23"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A4:B4"/>

</xml_diff>